<commit_message>
Ships recalibrated as domestic only
</commit_message>
<xml_diff>
--- a/InputData/trans/BNVFE/BAU New Veh Fuel Economy.xlsx
+++ b/InputData/trans/BNVFE/BAU New Veh Fuel Economy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\BNVFE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0295E1B5-04B4-495D-BAC3-233A5CC68C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BC1A94-0FBE-4037-A2D4-66A4923CE019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28050" yWindow="1860" windowWidth="27045" windowHeight="14940" activeTab="1" xr2:uid="{D850E225-7E57-43A0-BCF6-AD6641E8498D}"/>
+    <workbookView xWindow="-26580" yWindow="750" windowWidth="25050" windowHeight="14940" firstSheet="23" activeTab="27" xr2:uid="{D850E225-7E57-43A0-BCF6-AD6641E8498D}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -10996,16 +10996,16 @@
         <v>20</v>
       </c>
       <c r="B6" s="34">
-        <v>1.3426499999999999E-2</v>
+        <v>2.8195999999999998E-3</v>
       </c>
       <c r="C6" s="34">
         <v>0</v>
       </c>
       <c r="D6" s="34">
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="E6" s="34">
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -11014,7 +11014,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="34">
-        <v>1.25346E-2</v>
+        <v>2.6323000000000002E-3</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -19376,127 +19376,127 @@
       </c>
       <c r="B2" s="13">
         <f>B5*Calibration!$B$43</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="C2" s="13">
         <f>B2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="D2" s="13">
         <f>C2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="E2" s="13">
         <f>D2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="F2" s="13">
         <f>E2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="G2" s="13">
         <f>F2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="H2" s="13">
         <f>G2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="I2" s="13">
         <f>H2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="J2" s="13">
         <f>I2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="K2" s="13">
         <f>J2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="L2" s="13">
         <f>K2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="M2" s="13">
         <f>L2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="N2" s="13">
         <f>M2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="O2" s="13">
         <f>N2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="P2" s="13">
         <f>O2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="Q2" s="13">
         <f>P2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="R2" s="13">
         <f>Q2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="S2" s="13">
         <f>R2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="T2" s="13">
         <f>S2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="U2" s="13">
         <f>T2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="V2" s="13">
         <f>U2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="W2" s="13">
         <f>V2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="X2" s="13">
         <f>W2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="Y2" s="13">
         <f>X2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="Z2" s="13">
         <f>Y2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AA2" s="13">
         <f>Z2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AB2" s="13">
         <f>AA2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AC2" s="13">
         <f>AB2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AD2" s="13">
         <f>AC2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AE2" s="13">
         <f>AD2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
       <c r="AF2" s="13">
         <f>AE2*(1+CAGR!$C$58)</f>
-        <v>1.3426539742619228E-2</v>
+        <v>2.8195026495079485E-3</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -19634,127 +19634,127 @@
       </c>
       <c r="B4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="C4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="D4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="E4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="F4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="G4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="H4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="I4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="J4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="K4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="L4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="M4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="N4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="O4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="P4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Q4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="R4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="S4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="T4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="U4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="V4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="W4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="X4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Y4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Z4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AA4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AB4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AC4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AD4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AE4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AF4">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A4,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A4,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
     </row>
     <row r="5" spans="1:32">
@@ -19763,127 +19763,127 @@
       </c>
       <c r="B5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="C5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="D5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="E5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="F5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="G5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="H5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="I5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="J5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="K5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="L5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="M5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="N5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="O5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="P5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Q5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="R5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="S5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="T5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="U5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="V5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="W5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="X5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Y5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="Z5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AA5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AB5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AC5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AD5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AE5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
       <c r="AF5" s="14">
         <f>IFERROR(INDEX('SYFAFE psgr'!$B$6:$H$6,,MATCH($A5,'SYFAFE psgr'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$58:$C$64,MATCH($A5,CAGR!$B$58:$B$64,0))),0)</f>
-        <v>4.1782E-3</v>
+        <v>8.7739999999999997E-4</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -20150,127 +20150,127 @@
       </c>
       <c r="B8" s="13">
         <f>B5*Calibration!D43</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="C8" s="13">
         <f>B8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="D8" s="13">
         <f>C8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="E8" s="13">
         <f>D8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="F8" s="13">
         <f>E8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="G8" s="13">
         <f>F8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="H8" s="13">
         <f>G8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="I8" s="13">
         <f>H8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="J8" s="13">
         <f>I8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="K8" s="13">
         <f>J8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="L8" s="13">
         <f>K8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="M8" s="13">
         <f>L8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="N8" s="13">
         <f>M8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="O8" s="13">
         <f>N8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="P8" s="13">
         <f>O8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="Q8" s="13">
         <f>P8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="R8" s="13">
         <f>Q8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="S8" s="13">
         <f>R8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="T8" s="13">
         <f>S8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="U8" s="13">
         <f>T8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="V8" s="13">
         <f>U8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="W8" s="13">
         <f>V8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="X8" s="13">
         <f>W8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="Y8" s="13">
         <f>X8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="Z8" s="13">
         <f>Y8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AA8" s="13">
         <f>Z8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AB8" s="13">
         <f>AA8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AC8" s="13">
         <f>AB8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AD8" s="13">
         <f>AC8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AE8" s="13">
         <f>AD8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
       <c r="AF8" s="13">
         <f>AE8*(1+CAGR!$C$64)</f>
-        <v>1.2534599999999998E-2</v>
+        <v>2.6321999999999995E-3</v>
       </c>
     </row>
   </sheetData>
@@ -20394,127 +20394,127 @@
       </c>
       <c r="B2" s="13">
         <f>B5*Calibration!$B$44</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="C2" s="13">
         <f>B2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="D2" s="13">
         <f>C2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="E2" s="13">
         <f>D2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="F2" s="13">
         <f>E2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="G2" s="13">
         <f>F2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="H2" s="13">
         <f>G2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="I2" s="13">
         <f>H2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="J2" s="13">
         <f>I2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="K2" s="13">
         <f>J2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="L2" s="13">
         <f>K2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="M2" s="13">
         <f>L2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="N2" s="13">
         <f>M2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="O2" s="13">
         <f>N2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="P2" s="13">
         <f>O2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="Q2" s="13">
         <f>P2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="R2" s="13">
         <f>Q2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="S2" s="13">
         <f>R2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="T2" s="13">
         <f>S2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="U2" s="13">
         <f>T2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="V2" s="13">
         <f>U2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="W2" s="13">
         <f>V2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="X2" s="13">
         <f>W2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="Y2" s="13">
         <f>X2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="Z2" s="13">
         <f>Y2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AA2" s="13">
         <f>Z2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AB2" s="13">
         <f>AA2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AC2" s="13">
         <f>AB2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AD2" s="13">
         <f>AC2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AE2" s="13">
         <f>AD2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
       <c r="AF2" s="13">
         <f>AE2*(1+CAGR!$C$65)</f>
-        <v>1.5613951930355792E-2</v>
+        <v>3.2790295230885696E-3</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -20523,127 +20523,127 @@
       </c>
       <c r="B3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$65:$C$71,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="C3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="D3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="E3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="F3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="G3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="H3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="I3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="J3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="K3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="L3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="M3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="N3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="O3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="P3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Q3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="R3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="S3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="T3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="U3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="V3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="W3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="X3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Y3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Z3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AA3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AB3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AC3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AD3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AE3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AF3">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A3,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A3,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
     </row>
     <row r="4" spans="1:32">
@@ -20652,127 +20652,127 @@
       </c>
       <c r="B4" s="14">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A4,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$65:$C$71,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="C4" s="14">
         <f>IFERROR(B4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="D4" s="14">
         <f>IFERROR(C4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="E4" s="14">
         <f>IFERROR(D4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="F4" s="14">
         <f>IFERROR(E4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="G4" s="14">
         <f>IFERROR(F4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="H4" s="14">
         <f>IFERROR(G4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="I4" s="14">
         <f>IFERROR(H4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="J4" s="14">
         <f>IFERROR(I4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="K4" s="14">
         <f>IFERROR(J4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="L4" s="14">
         <f>IFERROR(K4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="M4" s="14">
         <f>IFERROR(L4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="N4" s="14">
         <f>IFERROR(M4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="O4" s="14">
         <f>IFERROR(N4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="P4" s="14">
         <f>IFERROR(O4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Q4" s="14">
         <f>IFERROR(P4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="R4" s="14">
         <f>IFERROR(Q4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="S4" s="14">
         <f>IFERROR(R4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="T4" s="14">
         <f>IFERROR(S4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="U4" s="14">
         <f>IFERROR(T4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="V4" s="14">
         <f>IFERROR(U4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="W4" s="14">
         <f>IFERROR(V4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="X4" s="14">
         <f>IFERROR(W4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Y4" s="14">
         <f>IFERROR(X4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="Z4" s="14">
         <f>IFERROR(Y4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AA4" s="14">
         <f>IFERROR(Z4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AB4" s="14">
         <f>IFERROR(AA4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AC4" s="14">
         <f>IFERROR(AB4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AD4" s="14">
         <f>IFERROR(AC4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AE4" s="14">
         <f>IFERROR(AD4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="AF4" s="14">
         <f>IFERROR(AE4*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A4,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
     </row>
     <row r="5" spans="1:32">
@@ -20781,127 +20781,127 @@
       </c>
       <c r="B5" s="14">
         <f>IFERROR(INDEX('SYFAFE frgt'!$B$6:$H$6,,MATCH($A5,'SYFAFE frgt'!$B$1:$H$1,0))*(1+INDEX(CAGR!$C$65:$C$71,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="C5" s="14">
         <f>IFERROR(B5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.8893954176843649E-3</v>
+        <v>1.0268042322758497E-3</v>
       </c>
       <c r="D5" s="14">
         <f>IFERROR(C5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.9200822306433275E-3</v>
+        <v>1.0332486587804753E-3</v>
       </c>
       <c r="E5" s="14">
         <f>IFERROR(D5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.950961640111497E-3</v>
+        <v>1.0397335317808088E-3</v>
       </c>
       <c r="F5" s="14">
         <f>IFERROR(E5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>4.9820348548626683E-3</v>
+        <v>1.0462591051270589E-3</v>
       </c>
       <c r="G5" s="14">
         <f>IFERROR(F5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.0133030912571401E-3</v>
+        <v>1.052825634262649E-3</v>
       </c>
       <c r="H5" s="14">
         <f>IFERROR(G5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.0447675732893287E-3</v>
+        <v>1.0594333762342157E-3</v>
       </c>
       <c r="I5" s="14">
         <f>IFERROR(H5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.0764295326356816E-3</v>
+        <v>1.0660825897016711E-3</v>
       </c>
       <c r="J5" s="14">
         <f>IFERROR(I5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.1082902087028915E-3</v>
+        <v>1.072773534948328E-3</v>
       </c>
       <c r="K5" s="14">
         <f>IFERROR(J5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.1403508486764131E-3</v>
+        <v>1.079506473891089E-3</v>
       </c>
       <c r="L5" s="14">
         <f>IFERROR(K5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.1726127075692827E-3</v>
+        <v>1.0862816700906988E-3</v>
       </c>
       <c r="M5" s="14">
         <f>IFERROR(L5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.205077048271247E-3</v>
+        <v>1.0930993887620615E-3</v>
       </c>
       <c r="N5" s="14">
         <f>IFERROR(M5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.2377451415981996E-3</v>
+        <v>1.0999598967846227E-3</v>
       </c>
       <c r="O5" s="14">
         <f>IFERROR(N5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.2706182663419246E-3</v>
+        <v>1.1068634627128158E-3</v>
       </c>
       <c r="P5" s="14">
         <f>IFERROR(O5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.3036977093201577E-3</v>
+        <v>1.1138103567865751E-3</v>
       </c>
       <c r="Q5" s="14">
         <f>IFERROR(P5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.3369847654269565E-3</v>
+        <v>1.1208008509419143E-3</v>
       </c>
       <c r="R5" s="14">
         <f>IFERROR(Q5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.3704807376833896E-3</v>
+        <v>1.1278352188215711E-3</v>
       </c>
       <c r="S5" s="14">
         <f>IFERROR(R5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.4041869372885446E-3</v>
+        <v>1.1349137357857194E-3</v>
       </c>
       <c r="T5" s="14">
         <f>IFERROR(S5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.4381046836708535E-3</v>
+        <v>1.142036678922748E-3</v>
       </c>
       <c r="U5" s="14">
         <f>IFERROR(T5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.4722353045397413E-3</v>
+        <v>1.1492043270601071E-3</v>
       </c>
       <c r="V5" s="14">
         <f>IFERROR(U5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.506580135937602E-3</v>
+        <v>1.156416960775223E-3</v>
       </c>
       <c r="W5" s="14">
         <f>IFERROR(V5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.5411405222920941E-3</v>
+        <v>1.1636748624064819E-3</v>
       </c>
       <c r="X5" s="14">
         <f>IFERROR(W5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.5759178164687707E-3</v>
+        <v>1.1709783160642811E-3</v>
       </c>
       <c r="Y5" s="14">
         <f>IFERROR(X5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.6109133798240372E-3</v>
+        <v>1.1783276076421515E-3</v>
       </c>
       <c r="Z5" s="14">
         <f>IFERROR(Y5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.6461285822584405E-3</v>
+        <v>1.1857230248279477E-3</v>
       </c>
       <c r="AA5" s="14">
         <f>IFERROR(Z5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.6815648022702945E-3</v>
+        <v>1.1931648571151107E-3</v>
       </c>
       <c r="AB5" s="14">
         <f>IFERROR(AA5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.7172234270096425E-3</v>
+        <v>1.2006533958139993E-3</v>
       </c>
       <c r="AC5" s="14">
         <f>IFERROR(AB5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.7531058523325532E-3</v>
+        <v>1.2081889340632942E-3</v>
       </c>
       <c r="AD5" s="14">
         <f>IFERROR(AC5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.7892134828557672E-3</v>
+        <v>1.2157717668414719E-3</v>
       </c>
       <c r="AE5" s="14">
         <f>IFERROR(AD5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.8255477320116747E-3</v>
+        <v>1.2234021909783522E-3</v>
       </c>
       <c r="AF5" s="14">
         <f>IFERROR(AE5*(1+INDEX(CAGR!$C$51:$C$57,MATCH($A5,CAGR!$B$65:$B$71,0))),0)</f>
-        <v>5.8621100221036499E-3</v>
+        <v>1.2310805051667182E-3</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -21168,127 +21168,127 @@
       </c>
       <c r="B8" s="13">
         <f>B5*Calibration!$D$44</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="C8" s="13">
         <f>B8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="D8" s="13">
         <f>C8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="E8" s="13">
         <f>D8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="F8" s="13">
         <f>E8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="G8" s="13">
         <f>F8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="H8" s="13">
         <f>G8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="I8" s="13">
         <f>H8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="J8" s="13">
         <f>I8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="K8" s="13">
         <f>J8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="L8" s="13">
         <f>K8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="M8" s="13">
         <f>L8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="N8" s="13">
         <f>M8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="O8" s="13">
         <f>N8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="P8" s="13">
         <f>O8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="Q8" s="13">
         <f>P8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="R8" s="13">
         <f>Q8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="S8" s="13">
         <f>R8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="T8" s="13">
         <f>S8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="U8" s="13">
         <f>T8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="V8" s="13">
         <f>U8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="W8" s="13">
         <f>V8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="X8" s="13">
         <f>W8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="Y8" s="13">
         <f>X8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="Z8" s="13">
         <f>Y8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AA8" s="13">
         <f>Z8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AB8" s="13">
         <f>AA8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AC8" s="13">
         <f>AB8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AD8" s="13">
         <f>AC8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AE8" s="13">
         <f>AD8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
       <c r="AF8" s="13">
         <f>AE8*(1+CAGR!$C$71)</f>
-        <v>1.4576699999999998E-2</v>
+        <v>3.0611999999999996E-3</v>
       </c>
     </row>
   </sheetData>
@@ -21460,16 +21460,16 @@
         <v>20</v>
       </c>
       <c r="B6" s="34">
-        <v>1.5614100000000001E-2</v>
+        <v>3.2789999999999998E-3</v>
       </c>
       <c r="C6" s="34">
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="D6" s="34">
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="E6" s="34">
-        <v>4.8589000000000002E-3</v>
+        <v>1.0204000000000001E-3</v>
       </c>
       <c r="F6" s="34">
         <v>0</v>
@@ -21478,7 +21478,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="34">
-        <v>1.4576799999999999E-2</v>
+        <v>3.0611000000000002E-3</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>

</xml_diff>